<commit_message>
Remove target exit, recompute with 45 strategies
- Removed Exit_Target (3% profit target) exit criterion
- Now 9 exit variations (5 RSI thresholds + 4 new methods)
- Total 45 strategy combinations (5 entries x 9 exits)
- Top performer: Entry_10_Exit_RSI_75 with PF 19.06
- Created ftd_table2.xlsx and ftd_performance2.png

Co-authored-by: openhands <openhands@all-hands.dev>
</commit_message>
<xml_diff>
--- a/ftd_table2.xlsx
+++ b/ftd_table2.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -475,1248 +475,1123 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Target</t>
+          <t>Entry_10_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>316.75%</t>
+          <t>236.93%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>7.77</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>55.6%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_Target</t>
+          <t>Entry_10_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>247.86%</t>
+          <t>264.42%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>7.64</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>87.2%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Target</t>
+          <t>Entry_10_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>157.67%</t>
+          <t>202.91%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>6.41</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>87.5%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Target</t>
+          <t>Entry_10_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>59.36%</t>
+          <t>136.51%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>inf</t>
+          <t>6.30</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>90.2%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_Oversold</t>
+          <t>Entry_10_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>236.93%</t>
+          <t>155.63%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>7.77</t>
+          <t>5.65</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>87.8%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_70</t>
+          <t>Entry_15_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>264.42%</t>
+          <t>47.34%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>7.64</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>87.2%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_65</t>
+          <t>Entry_7_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>202.91%</t>
+          <t>186.23%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>6.41</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_55</t>
+          <t>Entry_10_Exit_Time_10</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>136.51%</t>
+          <t>84.87%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>6.30</t>
+          <t>3.41</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>90.2%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_60</t>
+          <t>Entry_7_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>155.63%</t>
+          <t>213.67%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5.65</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>88.1%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_65</t>
+          <t>Entry_8_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>47.34%</t>
+          <t>113.57%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>3.94</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>76.3%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_60</t>
+          <t>Entry_7_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>186.23%</t>
+          <t>189.16%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.16</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>80.4%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_Time_10</t>
+          <t>Entry_7_Exit_Time_3</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>84.87%</t>
+          <t>119.25%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>3.41</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>74.6%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_75</t>
+          <t>Entry_10_Exit_Time_3</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>213.66%</t>
+          <t>63.14%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>2.94</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>88.1%</t>
+          <t>77.4%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_60</t>
+          <t>Entry_7_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>113.57%</t>
+          <t>87.38%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>2.83</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>72.0%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_65</t>
+          <t>Entry_7_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>189.16%</t>
+          <t>133.22%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>77.6%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Time_3</t>
+          <t>Entry_8_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>119.25%</t>
+          <t>96.63%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>2.63</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>74.3%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_Target</t>
+          <t>Entry_10_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>296.33%</t>
+          <t>42.42%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>283.67</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>97.6%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_Time_3</t>
+          <t>Entry_8_Exit_Time_3</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>63.14%</t>
+          <t>65.22%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2.94</t>
+          <t>2.58</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>77.4%</t>
+          <t>73.9%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_MA_Cross</t>
+          <t>Entry_15_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>87.38%</t>
+          <t>29.76%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2.83</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_55</t>
+          <t>Entry_7_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>133.22%</t>
+          <t>153.37%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>81.8%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_65</t>
+          <t>Entry_7_Exit_Time_10</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>96.63%</t>
+          <t>96.65%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>74.3%</t>
+          <t>64.8%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_MA_Cross</t>
+          <t>Entry_5_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>42.42%</t>
+          <t>142.32%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>80.3%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Time_3</t>
+          <t>Entry_8_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>65.22%</t>
+          <t>69.68%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2.58</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>73.9%</t>
+          <t>76.3%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_60</t>
+          <t>Entry_8_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>29.76%</t>
+          <t>53.89%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>81.5%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_70</t>
+          <t>Entry_10_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>153.37%</t>
+          <t>316.72%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>19.06</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>81.8%</t>
+          <t>89.5%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Time_10</t>
+          <t>Entry_5_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>96.65%</t>
+          <t>116.21%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>75.6%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_75</t>
+          <t>Entry_7_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>142.32%</t>
+          <t>78.42%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>80.3%</t>
+          <t>52.7%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_55</t>
+          <t>Entry_5_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>69.68%</t>
+          <t>99.67%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>79.2%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_75</t>
+          <t>Entry_15_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>53.89%</t>
+          <t>20.32%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>81.5%</t>
+          <t>84.6%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_75</t>
+          <t>Entry_5_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>316.72%</t>
+          <t>107.04%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>19.05</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>89.5%</t>
+          <t>73.6%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_65</t>
+          <t>Entry_8_Exit_Time_10</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>116.21%</t>
+          <t>43.39%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>64.3%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_Oversold</t>
+          <t>Entry_8_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>78.42%</t>
+          <t>38.44%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>52.7%</t>
+          <t>74.2%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_70</t>
+          <t>Entry_5_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>99.67%</t>
+          <t>71.59%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_75</t>
+          <t>Entry_15_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>20.32%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_60</t>
+          <t>Entry_15_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>107.04%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>73.6%</t>
+          <t>78.6%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Time_10</t>
+          <t>Entry_5_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>42</v>
+        <v>154</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>43.39%</t>
+          <t>55.42%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>34.4%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_70</t>
+          <t>Entry_15_Exit_Time_3</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>38.44%</t>
+          <t>1.96%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>74.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_55</t>
+          <t>Entry_8_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>71.59%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>26.0%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_55</t>
+          <t>Entry_8_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>2.05%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>49.1%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_70</t>
+          <t>Entry_15_Exit_Time_10</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>-3.43%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>53.3%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_Oversold</t>
+          <t>Entry_5_Exit_Time_3</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>153</v>
+        <v>193</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>58.13%</t>
+          <t>-11.54%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>53.4%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Time_3</t>
+          <t>Entry_5_Exit_Time_10</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>15</v>
+        <v>122</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>1.96%</t>
+          <t>-20.61%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>56.6%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_Oversold</t>
+          <t>Entry_15_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>-2.72%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>43.8%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_MA_Cross</t>
+          <t>Entry_5_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>55</v>
+        <v>281</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>2.05%</t>
+          <t>-29.54%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>49.1%</t>
+          <t>43.1%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Time_10</t>
+          <t>Entry_15_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-7.27%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>53.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Entry_5_Exit_Time_3</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>192</v>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>-8.28%</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>53.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Entry_5_Exit_Time_10</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>122</v>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>-20.61%</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>0.97</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>56.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Entry_15_Exit_RSI_Oversold</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>-2.72%</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>0.94</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>43.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Entry_5_Exit_MA_Cross</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>-28.31%</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>0.89</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>43.2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Entry_15_Exit_MA_Cross</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>-7.27%</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>0.60</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>56.2%</t>
         </is>
@@ -1854,7 +1729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2032,23 +1907,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Exit_Target</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Exit when profit target of 3% is reached</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Profit Target</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add FTD comparison chart
- Create Entry_10_no_ftd entry condition for comparison
- Compare Entry_10_Exit_RSI_75 with FTD vs without FTD
- With FTD: 5 trades, 18.32% return, PF 4.48
- Without FTD: 38 trades, 316.72% return, PF 19.06
- Created ftd_comparison.png showing both equity curves

Co-authored-by: openhands <openhands@all-hands.dev>
</commit_message>
<xml_diff>
--- a/ftd_table2.xlsx
+++ b/ftd_table2.xlsx
@@ -479,903 +479,903 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>236.93%</t>
+          <t>27.79%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>7.77</t>
+          <t>7.70</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_70</t>
+          <t>Entry_10_Exit_Time_3</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>264.42%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>7.64</t>
+          <t>5.23</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>87.2%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_65</t>
+          <t>Entry_10_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>202.91%</t>
+          <t>18.32%</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>6.41</t>
+          <t>4.48</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_55</t>
+          <t>Entry_15_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>136.51%</t>
+          <t>47.34%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>6.30</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>90.2%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_60</t>
+          <t>Entry_7_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>155.63%</t>
+          <t>186.23%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>5.65</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>87.8%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_65</t>
+          <t>Entry_7_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>47.34%</t>
+          <t>213.67%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>3.94</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>88.1%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_60</t>
+          <t>Entry_8_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>186.23%</t>
+          <t>113.57%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.19</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>76.3%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_Time_10</t>
+          <t>Entry_7_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>84.87%</t>
+          <t>189.16%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>3.41</t>
+          <t>3.16</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>80.4%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_75</t>
+          <t>Entry_7_Exit_Time_3</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>213.67%</t>
+          <t>119.25%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>88.1%</t>
+          <t>74.6%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_60</t>
+          <t>Entry_7_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>113.57%</t>
+          <t>87.38%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>2.83</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>72.0%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_65</t>
+          <t>Entry_7_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>189.16%</t>
+          <t>133.22%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>77.6%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Time_3</t>
+          <t>Entry_8_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>119.25%</t>
+          <t>96.63%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>2.63</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>74.3%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_Time_3</t>
+          <t>Entry_8_Exit_Time_3</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>63.14%</t>
+          <t>65.22%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2.94</t>
+          <t>2.58</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>77.4%</t>
+          <t>73.9%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_MA_Cross</t>
+          <t>Entry_7_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>87.38%</t>
+          <t>153.37%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2.83</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>81.8%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_55</t>
+          <t>Entry_15_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>133.22%</t>
+          <t>29.76%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_65</t>
+          <t>Entry_7_Exit_Time_10</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>96.63%</t>
+          <t>96.65%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>74.3%</t>
+          <t>64.8%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_MA_Cross</t>
+          <t>Entry_5_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>42.42%</t>
+          <t>142.32%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>80.3%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Time_3</t>
+          <t>Entry_8_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>65.22%</t>
+          <t>69.68%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2.58</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>73.9%</t>
+          <t>76.3%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_60</t>
+          <t>Entry_8_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>29.76%</t>
+          <t>53.89%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>81.5%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_70</t>
+          <t>Entry_5_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>153.37%</t>
+          <t>116.21%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>81.8%</t>
+          <t>75.6%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Time_10</t>
+          <t>Entry_7_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>96.65%</t>
+          <t>78.42%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>52.7%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_75</t>
+          <t>Entry_15_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>66</v>
+        <v>13</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>142.32%</t>
+          <t>20.32%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>80.3%</t>
+          <t>84.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_55</t>
+          <t>Entry_5_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>69.68%</t>
+          <t>99.67%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>79.2%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_75</t>
+          <t>Entry_5_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>53.89%</t>
+          <t>107.04%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>81.5%</t>
+          <t>73.6%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_75</t>
+          <t>Entry_8_Exit_Time_10</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>316.72%</t>
+          <t>43.39%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>19.06</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>89.5%</t>
+          <t>64.3%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_65</t>
+          <t>Entry_8_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>116.21%</t>
+          <t>38.44%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>74.2%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_Oversold</t>
+          <t>Entry_5_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>78.42%</t>
+          <t>71.59%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>52.7%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_70</t>
+          <t>Entry_10_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>72</v>
+        <v>5</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>99.67%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_75</t>
+          <t>Entry_15_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>20.32%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_60</t>
+          <t>Entry_15_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>107.04%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>73.6%</t>
+          <t>78.6%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Time_10</t>
+          <t>Entry_5_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>42</v>
+        <v>153</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>43.39%</t>
+          <t>58.14%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>34.6%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_70</t>
+          <t>Entry_15_Exit_Time_3</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>38.44%</t>
+          <t>1.96%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>74.2%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_55</t>
+          <t>Entry_8_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>71.59%</t>
+          <t>0.82%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>26.0%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_55</t>
+          <t>Entry_10_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>-0.24%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_70</t>
+          <t>Entry_8_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>14</v>
+        <v>55</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>2.05%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>49.1%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_Oversold</t>
+          <t>Entry_10_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>154</v>
+        <v>5</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>55.42%</t>
+          <t>-0.48%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>34.4%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Time_3</t>
+          <t>Entry_15_Exit_Time_10</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1383,217 +1383,217 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1.96%</t>
+          <t>-3.43%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>53.3%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_Oversold</t>
+          <t>Entry_10_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>-1.17%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_MA_Cross</t>
+          <t>Entry_10_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>2.05%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>49.1%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Time_10</t>
+          <t>Entry_5_Exit_Time_3</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>15</v>
+        <v>192</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-8.28%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>53.3%</t>
+          <t>53.6%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_Time_3</t>
+          <t>Entry_5_Exit_Time_10</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>193</v>
+        <v>122</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>-11.54%</t>
+          <t>-20.61%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>53.4%</t>
+          <t>56.6%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_Time_10</t>
+          <t>Entry_15_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>122</v>
+        <v>16</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>-20.61%</t>
+          <t>-2.72%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>0.97</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>56.6%</t>
+          <t>43.8%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_Oversold</t>
+          <t>Entry_5_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>16</v>
+        <v>280</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>-2.72%</t>
+          <t>-28.31%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>43.2%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_MA_Cross</t>
+          <t>Entry_15_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>281</v>
+        <v>16</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>-29.54%</t>
+          <t>-7.27%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>43.1%</t>
+          <t>56.2%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_MA_Cross</t>
+          <t>Entry_10_Exit_Time_10</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>-7.27%</t>
+          <t>-14.85%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>56.2%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Add FTD criteria to Entry_7 and Entry_8
- Entry_7 was missing FTD - only had RSI < 30 + Volume Spike
- Entry_8 was missing FTD - only had RSI < 30 + Gap Up
- Both now include: RSI < 30 + FTD + additional filter
- Trade counts dropped: Entry_7 (49->6), Entry_8 (38->12)
- All top 5 entries now include FTD as intended

Co-authored-by: openhands <openhands@all-hands.dev>
</commit_message>
<xml_diff>
--- a/ftd_table2.xlsx
+++ b/ftd_table2.xlsx
@@ -550,350 +550,350 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_65</t>
+          <t>Entry_7_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>47.34%</t>
+          <t>18.20%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>3.94</t>
+          <t>4.41</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_60</t>
+          <t>Entry_15_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>186.23%</t>
+          <t>47.34%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_75</t>
+          <t>Entry_8_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>213.67%</t>
+          <t>24.26%</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>88.1%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_60</t>
+          <t>Entry_8_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>113.57%</t>
+          <t>29.57%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>35.7%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_65</t>
+          <t>Entry_15_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>189.16%</t>
+          <t>29.76%</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Time_3</t>
+          <t>Entry_5_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>119.25%</t>
+          <t>140.86%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>74.6%</t>
+          <t>80.3%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_MA_Cross</t>
+          <t>Entry_8_Exit_Time_3</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>75</v>
+        <v>13</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>87.38%</t>
+          <t>11.91%</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2.83</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>69.2%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_55</t>
+          <t>Entry_5_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>133.22%</t>
+          <t>114.92%</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>74.4%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_65</t>
+          <t>Entry_15_Exit_RSI_75</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>96.63%</t>
+          <t>20.32%</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>74.3%</t>
+          <t>84.6%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Time_3</t>
+          <t>Entry_5_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>65.22%</t>
+          <t>98.47%</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2.58</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>73.9%</t>
+          <t>77.8%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_70</t>
+          <t>Entry_5_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>44</v>
+        <v>91</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>153.37%</t>
+          <t>105.80%</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>81.8%</t>
+          <t>72.5%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_60</t>
+          <t>Entry_8_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>29.76%</t>
+          <t>18.68%</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_Time_10</t>
+          <t>Entry_8_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>96.65%</t>
+          <t>14.59%</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>64.8%</t>
+          <t>63.6%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_75</t>
+          <t>Entry_5_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>142.32%</t>
+          <t>70.56%</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>80.3%</t>
+          <t>74.0%</t>
         </is>
       </c>
     </row>
@@ -904,253 +904,253 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>69.68%</t>
+          <t>11.47%</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>76.3%</t>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_75</t>
+          <t>Entry_10_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>53.89%</t>
+          <t>5.50%</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>81.5%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_65</t>
+          <t>Entry_8_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>116.21%</t>
+          <t>7.99%</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>75.6%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Entry_7_Exit_RSI_Oversold</t>
+          <t>Entry_15_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>78.42%</t>
+          <t>7.66%</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>52.7%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_75</t>
+          <t>Entry_15_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>20.32%</t>
+          <t>4.39%</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>78.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_70</t>
+          <t>Entry_5_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>72</v>
+        <v>153</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>99.67%</t>
+          <t>58.13%</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>79.2%</t>
+          <t>34.6%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_60</t>
+          <t>Entry_8_Exit_Time_10</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>91</v>
+        <v>13</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>107.04%</t>
+          <t>3.63%</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>73.6%</t>
+          <t>53.8%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_Time_10</t>
+          <t>Entry_7_Exit_RSI_70</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>43.39%</t>
+          <t>1.80%</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>64.3%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_70</t>
+          <t>Entry_7_Exit_Time_3</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>38.44%</t>
+          <t>0.74%</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>74.2%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_55</t>
+          <t>Entry_15_Exit_Time_3</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>96</v>
+        <v>15</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>71.59%</t>
+          <t>1.96%</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_70</t>
+          <t>Entry_10_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -1158,149 +1158,149 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>5.50%</t>
+          <t>-0.24%</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_55</t>
+          <t>Entry_10_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>7.66%</t>
+          <t>-0.48%</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_70</t>
+          <t>Entry_15_Exit_Time_10</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>4.39%</t>
+          <t>-3.43%</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>53.3%</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_RSI_Oversold</t>
+          <t>Entry_10_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>153</v>
+        <v>5</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>58.14%</t>
+          <t>-1.17%</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Time_3</t>
+          <t>Entry_7_Exit_RSI_60</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1.96%</t>
+          <t>-1.28%</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_RSI_Oversold</t>
+          <t>Entry_5_Exit_Time_3</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>50</v>
+        <v>193</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>0.82%</t>
+          <t>-9.82%</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>53.4%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_55</t>
+          <t>Entry_10_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -1308,292 +1308,292 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>-0.24%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Entry_8_Exit_MA_Cross</t>
+          <t>Entry_5_Exit_Time_10</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>55</v>
+        <v>123</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2.05%</t>
+          <t>-23.10%</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>49.1%</t>
+          <t>56.1%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_65</t>
+          <t>Entry_15_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>-0.48%</t>
+          <t>-2.72%</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>43.8%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_Time_10</t>
+          <t>Entry_7_Exit_RSI_65</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>-3.43%</t>
+          <t>-2.54%</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>53.3%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_RSI_60</t>
+          <t>Entry_5_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>5</v>
+        <v>281</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>-1.17%</t>
+          <t>-28.52%</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>43.1%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_MA_Cross</t>
+          <t>Entry_8_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>-0.09%</t>
+          <t>-4.35%</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>60.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_Time_3</t>
+          <t>Entry_7_Exit_RSI_55</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>192</v>
+        <v>6</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>-8.28%</t>
+          <t>-5.95%</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.65</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>53.6%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_Time_10</t>
+          <t>Entry_15_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>122</v>
+        <v>16</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>-20.61%</t>
+          <t>-7.27%</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>0.97</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>56.6%</t>
+          <t>56.2%</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_RSI_Oversold</t>
+          <t>Entry_10_Exit_Time_10</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>-2.72%</t>
+          <t>-14.85%</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>43.8%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Entry_5_Exit_MA_Cross</t>
+          <t>Entry_7_Exit_Time_10</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>280</v>
+        <v>6</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>-28.31%</t>
+          <t>-21.16%</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>43.2%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Entry_15_Exit_MA_Cross</t>
+          <t>Entry_7_Exit_MA_Cross</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>-7.27%</t>
+          <t>-7.56%</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>56.2%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Entry_10_Exit_Time_10</t>
+          <t>Entry_7_Exit_RSI_Oversold</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>-14.85%</t>
+          <t>-14.41%</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FTD vs No-FTD comparison
- Run all strategies WITH FTD and WITHOUT FTD criteria
- Excel now has perf_with_FTD and perf_no_FTD sheets
- Entry_15 updated to include FTD
- Added entry_condition_15_no_ftd for comparison
- Total 45 strategies for each version

Co-authored-by: openhands <openhands@all-hands.dev>
</commit_message>
<xml_diff>
--- a/ftd_table2.xlsx
+++ b/ftd_table2.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Perf" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Entries" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Exits" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="perf_with_FTD" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="perf_no_FTD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Entries" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Exits" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,7 +47,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,22 +55,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,13 +431,6 @@
   </sheetPr>
   <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -473,1125 +460,1125 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Entry_10_Exit_RSI_Oversold</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>27.79%</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>7.70</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>40.0%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Entry_10_Exit_Time_3</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" t="n">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>9.21%</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>5.23</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Entry_10_Exit_RSI_75</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>18.32%</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>4.48</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Entry_7_Exit_RSI_75</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" t="n">
         <v>6</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>18.20%</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>4.41</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>83.3%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Entry_15_Exit_RSI_65</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" t="n">
         <v>15</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>47.34%</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>3.94</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Entry_8_Exit_RSI_75</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>24.26%</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>2.46</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Entry_8_Exit_RSI_Oversold</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" t="n">
         <v>14</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>29.57%</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>2.45</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>35.7%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Entry_15_Exit_RSI_60</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" t="n">
         <v>15</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>29.76%</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>2.40</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Entry_5_Exit_RSI_75</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" t="n">
         <v>66</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>140.86%</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>142.32%</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2.21</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>80.3%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Entry_8_Exit_Time_3</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" t="n">
         <v>13</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>11.91%</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>2.03</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>69.2%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Entry_5_Exit_RSI_65</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" t="n">
         <v>82</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>114.92%</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>116.21%</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>1.85</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>74.4%</t>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>75.6%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Entry_15_Exit_RSI_75</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" t="n">
         <v>13</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>20.32%</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>1.80</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>84.6%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Entry_5_Exit_RSI_70</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" t="n">
         <v>72</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>98.47%</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>99.67%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>1.80</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>77.8%</t>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>79.2%</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Entry_5_Exit_RSI_60</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" t="n">
         <v>91</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>105.80%</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>107.04%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>1.79</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>72.5%</t>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>73.6%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Entry_8_Exit_RSI_60</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>18.68%</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>1.76</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Entry_8_Exit_RSI_65</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" t="n">
         <v>11</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>14.59%</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>1.63</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>63.6%</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Entry_5_Exit_RSI_55</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" t="n">
         <v>96</v>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>70.56%</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>71.59%</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>1.52</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>74.0%</t>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>75.0%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Entry_8_Exit_RSI_55</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" t="n">
         <v>12</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>11.47%</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>1.47</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>75.0%</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Entry_10_Exit_RSI_70</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" t="n">
         <v>5</v>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>5.50%</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Entry_8_Exit_RSI_70</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" t="n">
         <v>10</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>7.99%</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>1.37</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Entry_15_Exit_RSI_55</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>7.66%</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>1.34</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Entry_15_Exit_RSI_70</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B23" t="n">
         <v>14</v>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>4.39%</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>1.30</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>78.6%</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Entry_5_Exit_RSI_Oversold</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B24" t="n">
         <v>153</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>58.13%</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>1.27</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>34.6%</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Entry_8_Exit_Time_10</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B25" t="n">
         <v>13</v>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>3.63%</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>1.22</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>53.8%</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Entry_7_Exit_RSI_70</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B26" t="n">
         <v>6</v>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>1.80%</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>1.19</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Entry_7_Exit_Time_3</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B27" t="n">
         <v>6</v>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>0.74%</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>1.16</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Entry_15_Exit_Time_3</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" t="n">
         <v>15</v>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>1.96%</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>1.15</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Entry_10_Exit_RSI_55</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B29" t="n">
         <v>5</v>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>-0.24%</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>-0.23%</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>1.09</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>80.0%</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Entry_10_Exit_RSI_65</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B30" t="n">
         <v>5</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>-0.48%</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>1.05</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Entry_15_Exit_Time_10</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B31" t="n">
         <v>15</v>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>-3.43%</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>1.03</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>53.3%</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Entry_10_Exit_RSI_60</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B32" t="n">
         <v>5</v>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>-1.17%</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>1.02</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Entry_7_Exit_RSI_60</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B33" t="n">
         <v>6</v>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>-1.28%</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>1.01</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Entry_5_Exit_Time_3</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
-        <v>193</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>-9.82%</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="B34" t="n">
+        <v>192</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>-8.28%</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>53.4%</t>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>53.6%</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Entry_10_Exit_MA_Cross</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B35" t="n">
         <v>5</v>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>-0.09%</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>1.00</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Entry_5_Exit_Time_10</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
-        <v>123</v>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>-23.10%</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>0.95</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>56.1%</t>
+      <c r="B36" t="n">
+        <v>122</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>-20.61%</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>56.6%</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Entry_15_Exit_RSI_Oversold</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B37" t="n">
         <v>16</v>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>-2.72%</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>0.94</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>43.8%</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Entry_7_Exit_RSI_65</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
+      <c r="B38" t="n">
         <v>6</v>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>-2.54%</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>0.90</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Entry_5_Exit_MA_Cross</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>281</v>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>-28.52%</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="B39" t="n">
+        <v>280</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>-28.31%</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>0.89</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>43.1%</t>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>43.2%</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Entry_8_Exit_MA_Cross</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B40" t="n">
         <v>14</v>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>-4.35%</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>0.72</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Entry_7_Exit_RSI_55</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B41" t="n">
         <v>6</v>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>-5.95%</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>0.65</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>66.7%</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Entry_15_Exit_MA_Cross</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B42" t="n">
         <v>16</v>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>-7.27%</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>0.60</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>56.2%</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Entry_10_Exit_Time_10</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B43" t="n">
         <v>5</v>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>-14.85%</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>0.57</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>40.0%</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Entry_7_Exit_Time_10</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
+      <c r="B44" t="n">
         <v>6</v>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>-21.16%</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>0.26</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>33.3%</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Entry_7_Exit_MA_Cross</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
+      <c r="B45" t="n">
         <v>6</v>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>-7.56%</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>0.23</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>33.3%</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Entry_7_Exit_RSI_Oversold</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
+      <c r="B46" t="n">
         <v>6</v>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>-14.41%</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>0.00</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -1608,13 +1595,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1624,97 +1606,1147 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Num_Trades</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Total_Return</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Profit_Factor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Win_Rate</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Entry_10</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>RSI &lt; 30 + FTD + Price above 200-day MA (Trend Confirmation)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>FTD Entry</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_RSI_Oversold</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>579.25%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Entry_15</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>RSI &lt; 30 + FTD + Large green bar (&gt;1.5%) (Wide Bar)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>FTD Entry</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_RSI_Oversold</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>236.93%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>7.77</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>55.6%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Entry_7</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>RSI &lt; 30 + FTD + Volume &gt; 1.5x average (Volume Spike)</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>FTD Entry</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_RSI_70</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>264.42%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7.64</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>87.2%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Entry_8</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>RSI &lt; 30 + FTD + Gap up &gt; 0.5% (Gap Up)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>FTD Entry</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_RSI_65</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>40</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>202.91%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>6.41</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>87.5%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Entry_5</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>RSI &lt; 40 + FTD (IBS &gt; 0.5, any positive return)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>FTD Entry</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_RSI_55</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>41</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>136.51%</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>6.30</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>90.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_RSI_60</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>41</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>155.63%</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5.65</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>87.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_RSI_65</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>47.34%</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3.94</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>80.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_RSI_60</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>48</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>186.23%</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>83.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_Time_10</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>42</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>84.87%</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>3.41</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>66.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_RSI_75</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>42</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>213.66%</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>88.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_RSI_60</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>38</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>113.57%</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>3.19</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>76.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_RSI_65</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>46</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>189.16%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>80.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_Time_3</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>67</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>119.25%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>3.05</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>74.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_Time_3</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>53</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>63.14%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2.94</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>77.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_MA_Cross</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>75</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>87.38%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2.83</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>72.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_RSI_55</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>49</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>133.22%</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>77.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_RSI_65</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>35</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>96.63%</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2.63</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>74.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_MA_Cross</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>60</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>42.42%</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2.60</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>80.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_Time_3</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>46</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>65.22%</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2.58</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>73.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_RSI_75</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>80</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>281.53%</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2.49</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>81.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_RSI_70</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>44</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>153.37%</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>81.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_RSI_60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>15</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>29.76%</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>80.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_Time_10</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>54</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>96.65%</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>64.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_RSI_55</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>38</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>69.68%</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2.14</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>76.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_RSI_70</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>91</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>208.15%</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>80.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_RSI_75</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>27</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>53.89%</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>81.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_RSI_65</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>105</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>238.21%</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>78.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_RSI_60</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>120</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>233.32%</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>75.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Entry_10_Exit_RSI_75</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>38</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>316.72%</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>19.06</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>89.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_MA_Cross</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>269</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>399.70%</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1.98</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>70.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Entry_7_Exit_RSI_Oversold</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>55</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>78.42%</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>52.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_RSI_75</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>13</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>20.32%</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>84.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_RSI_55</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>134</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>172.66%</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>75.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_Time_10</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>42</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>43.39%</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>64.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_Time_10</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>135</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>163.25%</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1.64</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>65.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_RSI_70</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>31</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>38.44%</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>74.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Entry_5_Exit_Time_3</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>201</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>127.50%</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>69.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_RSI_55</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>15</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>7.66%</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>66.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_RSI_70</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>14</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>4.39%</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>78.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_Time_3</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>15</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1.96%</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>60.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_RSI_Oversold</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>50</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>0.82%</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>26.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Entry_8_Exit_MA_Cross</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>55</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2.05%</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>49.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_Time_10</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>15</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>-3.43%</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>53.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_RSI_Oversold</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>16</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>-2.72%</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>43.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Entry_15_Exit_MA_Cross</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>16</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>-7.27%</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>56.2%</t>
         </is>
       </c>
     </row>
@@ -1729,13 +2761,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1755,153 +2782,269 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Entry_10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RSI &lt; 30 + FTD + Price above 200-day MA (Trend Confirmation)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FTD Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Entry_15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RSI &lt; 30 + FTD + Large green bar (&gt;1.5%) (Wide Bar)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FTD Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Entry_7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RSI &lt; 30 + FTD + Volume &gt; 1.5x average (Volume Spike)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FTD Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Entry_8</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RSI &lt; 30 + FTD + Gap up &gt; 0.5% (Gap Up)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FTD Entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Entry_5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RSI &lt; 40 + FTD (IBS &gt; 0.5, any positive return)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FTD Entry</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Exit_RSI_55</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Exit when RSI &gt; 55</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>RSI Threshold</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Exit_RSI_60</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Exit when RSI &gt; 60</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>RSI Threshold</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Exit_RSI_65</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Exit when RSI &gt; 65</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>RSI Threshold</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Exit_RSI_70</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Exit when RSI &gt; 70</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>RSI Threshold</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Exit_RSI_75</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Exit when RSI &gt; 75</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>RSI Threshold</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Exit_Time_3</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Hold for 3 bars then exit</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Time-based</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Exit_Time_10</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Hold for 10 bars then exit</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Time-based</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Exit_RSI_Oversold</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Exit when RSI goes back below 30 (momentum fades)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>RSI Reversal</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Exit_MA_Cross</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Exit when price crosses below 20-day MA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>MA Cross</t>
         </is>

</xml_diff>